<commit_message>
투자 대시보드 2026-09-30 18:25
</commit_message>
<xml_diff>
--- a/technicals/exports/2026-09-29.xlsx
+++ b/technicals/exports/2026-09-29.xlsx
@@ -221,7 +221,7 @@
       </ns0:c>
       <ns0:c r="F3" t="inlineStr">
         <ns0:is>
-          <ns0:t>미충족 의료 수요를 위한 항체 의약품을 개발하며, 비호르몬성 혈관운동 증상 치료제를 임상 2상 중인 기업.</ns0:t>
+          <ns0:t>미충족 의료 수요 대상 항체 의약품을 개발하며 비호르몬성 혈관운동 증상 치료제 임상 2상을 진행하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G3">
@@ -300,7 +300,7 @@
       </ns0:c>
       <ns0:c r="F4" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국 뷰티·개인관리 브랜드에 전략, 마케팅, 전 채널 판매, 고객 서비스 및 물류 등 브랜드 관리 제공.</ns0:t>
+          <ns0:t>중국 뷰티·개인관리 브랜드에 전략·마케팅·전 채널 판매·고객 서비스·물류 등 브랜드 관리 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G4">
@@ -376,7 +376,7 @@
       </ns0:c>
       <ns0:c r="F5" t="inlineStr">
         <ns0:is>
-          <ns0:t>학교·가정·사무실·산업 시장 등에 절단·측정·응급처치·연마 제품을 공급하는 기업.</ns0:t>
+          <ns0:t>학교·가정·사무실·산업 시장에 절단·측정·응급처치·연마 제품을 공급하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G5">
@@ -455,7 +455,7 @@
       </ns0:c>
       <ns0:c r="F6" t="inlineStr">
         <ns0:is>
-          <ns0:t>북미·아시아태평양 등에서 전문·기술 컨설팅과 운영 모델 설계 관련 자문을 제공.</ns0:t>
+          <ns0:t>북미·아시아태평양 등에서 전문·기술 컨설팅과 운영 모델 설계 자문 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G6">
@@ -929,7 +929,7 @@
       </ns0:c>
       <ns0:c r="F12" t="inlineStr">
         <ns0:is>
-          <ns0:t>기업·공공부문 등에 컴퓨터 시스템과 데이터센터를 포함한 다양한 IT 솔루션을 제공하는 기업.</ns0:t>
+          <ns0:t>기업·공공부문에 컴퓨터 시스템·데이터센터 등 다양한 IT 솔루션을 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G12">
@@ -1245,7 +1245,7 @@
       </ns0:c>
       <ns0:c r="F16" t="inlineStr">
         <ns0:is>
-          <ns0:t>다중암 조기 발견 검사·서비스를 제공하며, 50세 초과 무증상자 대상 암 선별검사 Galleri를 공급하는 기업.</ns0:t>
+          <ns0:t>다중암 조기 발견 검사·서비스와 50세 초과 무증상자 대상 암 선별검사 Galleri를 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G16">
@@ -1400,7 +1400,7 @@
       </ns0:c>
       <ns0:c r="F18" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국과 해외에서 다양한 형태의 맞춤형 냉간 성형 강재를 제조·판매하는 회사.</ns0:t>
+          <ns0:t>중국과 해외에서 다양한 맞춤형 냉간 성형 강재를 제조·판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G18">
@@ -1479,7 +1479,7 @@
       </ns0:c>
       <ns0:c r="F19" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술로 의료 제공을 확장·자동화하며 급성 부상·만성 통증·수술 후 재활 등 근골격계 관리 플랫폼을 개발하는 기업.</ns0:t>
+          <ns0:t>급성 부상·만성 통증·수술 후 재활 등 근골격계 관리를 위한 의료 자동화 플랫폼 개발 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G19">
@@ -1558,7 +1558,7 @@
       </ns0:c>
       <ns0:c r="F20" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·영국 등에서 통신·결제 서비스를 제공하며 소매 솔루션·핀테크·Net2phone 사업 등을 운영하는 기업.</ns0:t>
+          <ns0:t>미국·영국 등에서 통신·결제 서비스를 제공하고 소매 솔루션·핀테크·Net2phone 사업 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G20">
@@ -1637,7 +1637,7 @@
       </ns0:c>
       <ns0:c r="F21" t="inlineStr">
         <ns0:is>
-          <ns0:t>유전·유전체 분석용 염기서열 분석 및 어레이 기반 장비와 소모품을 제공한다.</ns0:t>
+          <ns0:t>유전·유전체 분석용 염기서열 분석 및 어레이 기반 장비와 소모품 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G21">
@@ -1716,7 +1716,7 @@
       </ns0:c>
       <ns0:c r="F22" t="inlineStr">
         <ns0:is>
-          <ns0:t>전이성 흑색종과 기타 고형암 치료를 위한 자가 종양침윤림프구 기반 세포치료제를 개발·상용화한다.</ns0:t>
+          <ns0:t>전이성 흑색종·기타 고형암 치료용 자가 종양침윤림프구 기반 세포치료제 개발·상용화.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G22">
@@ -1795,7 +1795,7 @@
       </ns0:c>
       <ns0:c r="F23" t="inlineStr">
         <ns0:is>
-          <ns0:t>켄터키주에서 예금 등 다양한 은행 상품과 서비스를 제공하는 금융기관의 지주회사다.</ns0:t>
+          <ns0:t>켄터키주에서 예금 등 은행 상품과 서비스를 제공하는 금융기관의 지주회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G23">
@@ -1871,7 +1871,7 @@
       </ns0:c>
       <ns0:c r="F24" t="inlineStr">
         <ns0:is>
-          <ns0:t>보건·안전 분야에 사용하는 휴대용 질량분석기와 푸리에 변환 적외선 장비를 제공한다.</ns0:t>
+          <ns0:t>보건·안전 분야용 휴대용 질량분석기와 푸리에 변환 적외선 장비 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G24">
@@ -1950,7 +1950,7 @@
       </ns0:c>
       <ns0:c r="F25" t="inlineStr">
         <ns0:is>
-          <ns0:t>매립지 등 비화석연료원에서 바이오가스를 회수·처리하며 재생 천연가스와 재생 전력 사업을 한다.</ns0:t>
+          <ns0:t>매립지 등 비화석연료원의 바이오가스를 회수·처리하고 재생 천연가스·전력 사업 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G25">
@@ -2108,7 +2108,7 @@
       </ns0:c>
       <ns0:c r="F27" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 실험실용 기기 등 정밀기기를 제조·공급하고 관련 서비스를 제공한다.</ns0:t>
+          <ns0:t>전 세계에 실험실용 기기 등 정밀기기를 제조·공급하고 관련 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G27">
@@ -2187,7 +2187,7 @@
       </ns0:c>
       <ns0:c r="F28" t="inlineStr">
         <ns0:is>
-          <ns0:t>적층 제조 및 의료용 소프트웨어 도구와 3D 프린팅 서비스를 제공한다.</ns0:t>
+          <ns0:t>적층 제조·의료용 소프트웨어 도구와 3D 프린팅 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G28">
@@ -2266,7 +2266,7 @@
       </ns0:c>
       <ns0:c r="F29" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 기업 합병, 주식 교환, 자산 인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>주요 영업활동 없이 합병·주식 교환·자산 인수 등 기업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G29">
@@ -2342,7 +2342,7 @@
       </ns0:c>
       <ns0:c r="F30" t="inlineStr">
         <ns0:is>
-          <ns0:t>기업의 데이터 인프라 전환을 위한 소프트웨어, 시스템 및 서비스를 제공한다.</ns0:t>
+          <ns0:t>기업의 데이터 인프라 전환을 위한 소프트웨어·시스템·서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G30">
@@ -2421,7 +2421,7 @@
       </ns0:c>
       <ns0:c r="F31" t="inlineStr">
         <ns0:is>
-          <ns0:t>분자검사 서비스를 개발·상용화하며 미세잔존질환 평가, 재발 감시, 치료 반응 평가용 혈액검사를 제공한다.</ns0:t>
+          <ns0:t>분자검사를 개발·상용화하고 미세잔존질환·재발·치료 반응 평가용 혈액검사 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G31">
@@ -2500,7 +2500,7 @@
       </ns0:c>
       <ns0:c r="F32" t="inlineStr">
         <ns0:is>
-          <ns0:t>데이터 저장·관리 기술과 제품, 서비스를 제공하며 데이터 축소·보호·암호화 소프트웨어를 공급한다.</ns0:t>
+          <ns0:t>데이터 저장·관리 기술과 제품·서비스, 데이터 축소·보호·암호화 소프트웨어 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G32">
@@ -2579,7 +2579,7 @@
       </ns0:c>
       <ns0:c r="F33" t="inlineStr">
         <ns0:is>
-          <ns0:t>맞춤형 부품의 디지털 제조업체로 성형, CNC 가공, 3D 프린팅, 판금 제조 서비스를 제공한다.</ns0:t>
+          <ns0:t>맞춤형 부품의 디지털 제조업체로 성형·CNC 가공·3D 프린팅·판금 제조 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G33">
@@ -2658,7 +2658,7 @@
       </ns0:c>
       <ns0:c r="F34" t="inlineStr">
         <ns0:is>
-          <ns0:t>비정형 데이터 관리 솔루션과 영상 편집·후반 제작 등에 쓰이는 저장 소프트웨어 및 시스템을 제공한다.</ns0:t>
+          <ns0:t>비정형 데이터 관리 솔루션과 영상 편집·후반 제작용 저장 소프트웨어·시스템 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G34">
@@ -2737,7 +2737,7 @@
       </ns0:c>
       <ns0:c r="F35" t="inlineStr">
         <ns0:is>
-          <ns0:t>건강과학 분야의 장비·시약·소프트웨어와 검출·영상 기술, 질환 조기 탐지 솔루션을 제공한다.</ns0:t>
+          <ns0:t>건강과학 분야 장비·시약·소프트웨어와 검출·영상 기술, 질환 조기 탐지 솔루션 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G35">
@@ -2816,7 +2816,7 @@
       </ns0:c>
       <ns0:c r="F36" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 주요 안질환 치료를 위한 수술·비수술 기술을 개발하고 상용화하는 안과 의료기기 기업이다.</ns0:t>
+          <ns0:t>미국에서 주요 안질환 치료용 수술·비수술 기술을 개발·상용화하는 안과 의료기기 기업이다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G36">
@@ -2895,7 +2895,7 @@
       </ns0:c>
       <ns0:c r="F37" t="inlineStr">
         <ns0:is>
-          <ns0:t>서버 네트워크 인터페이스 카드와 암호화·압축용 카드 등 네트워크·데이터 인프라 솔루션을 설계·제조·판매.</ns0:t>
+          <ns0:t>서버 네트워크 인터페이스 카드와 암호화·압축용 카드 등 네트워크·데이터 인프라 솔루션을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G37">
@@ -3053,7 +3053,7 @@
       </ns0:c>
       <ns0:c r="F39" t="inlineStr">
         <ns0:is>
-          <ns0:t>자회사 Ctrl Media를 통해 홍콩에서 모바일 게임 앱 개발사 등에 통합 마케팅·광고 서비스를 제공.</ns0:t>
+          <ns0:t>자회사 Ctrl Media를 통해 홍콩에서 모바일 게임 앱 개발사 등에 통합 마케팅·광고를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G39">
@@ -3132,7 +3132,7 @@
       </ns0:c>
       <ns0:c r="F40" t="inlineStr">
         <ns0:is>
-          <ns0:t>선박 및 대형 비도로용 동력전달 장비를 설계·제조·판매하며 제조와 유통 부문을 운영한다.</ns0:t>
+          <ns0:t>선박·대형 비도로용 동력전달 장비를 설계·제조·판매하고 제조·유통 부문 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G40">
@@ -3211,7 +3211,7 @@
       </ns0:c>
       <ns0:c r="F41" t="inlineStr">
         <ns0:is>
-          <ns0:t>치료제·진단·소재·농업·데이터 저장·학술 연구 등에 쓰이는 합성 DNA 제품을 제조·판매한다.</ns0:t>
+          <ns0:t>치료제·진단·소재·농업·데이터 저장·학술 연구용 합성 DNA 제품 제조·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G41">
@@ -3527,7 +3527,7 @@
       </ns0:c>
       <ns0:c r="F45" t="inlineStr">
         <ns0:is>
-          <ns0:t>유의미한 영업활동 없이 기업 합병·주식 교환·자산 인수 등 사업결합을 추진한다.</ns0:t>
+          <ns0:t>유의미한 영업활동 없이 합병·주식 교환·자산 인수 등 사업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G45">
@@ -3682,7 +3682,7 @@
       </ns0:c>
       <ns0:c r="F47" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술 서비스 분야 기업과의 합병·주식 교환·자산 인수 등 사업결합을 추진한다.</ns0:t>
+          <ns0:t>기술 서비스 기업과의 합병·주식 교환·자산 인수 등 사업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G47">

</xml_diff>